<commit_message>
Added more filtering on the dashboard and a custom scraper to avoid google api fees (not fully optimized yet)
</commit_message>
<xml_diff>
--- a/places_to_call.xlsx
+++ b/places_to_call.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,16 @@
           <t>LastCallbackDate</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -503,6 +513,12 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -537,6 +553,12 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -563,6 +585,12 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -589,6 +617,12 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -615,6 +649,12 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -641,6 +681,12 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -667,6 +713,12 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -693,6 +745,12 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -719,6 +777,12 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -745,6 +809,1843 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>The Smokin' 116 Bistro</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>dont_call</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>(613) 902-5001</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>116 Pinnacle St, Belleville, ON K8N 3A4, Canada</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>weird mall type thing</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>(613) 902-5001</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Royal Haveli (Flavours of India)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>called</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>(613) 962-0043</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>366 N Front St #22, Belleville, ON K8P 5N8, Canada</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>left number for owner to callback on 2025-05-10</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>(613) 962-0043</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2025-05-10</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>The Pier Patio Bar and Grill</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>(613) 968-9494</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>1 S Front St, Belleville, ON K8N 5K7, Canada</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>was closed</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>(613) 968-9494</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2025-05-10</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Rosemary &amp; Thyme</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>(613) 962-9358</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>417 Bridge St E, Belleville, ON K8N 1P7, Canada</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>was closed</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>(613) 962-9358</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2025-05-10</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Toro Sushi Restaurant</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>called</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>(613) 967-6478</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>308 Dundas St E, Belleville, ON K8N 1E6, Canada</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>not interested : 2025-05-10</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>(613) 967-6478</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2025-05-10</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MAMA’S KITCHEN</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>(613) 779-7200</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>191 Dundas St E, Belleville, ON K8N 1E2, Canada</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>was closed</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>(613) 779-7200</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2025-05-10</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Harbour Cafe</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>(613) 966-8800</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>33 Pinnacle St, Belleville, ON K8N 3A1, Canada</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Heather's Place</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>(613) 771-1937</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>6835 ON-62, Belleville, ON K8N 0L9, Canada</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>OMG What a Hotdog!</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>(613) 779-7161</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>494 Dundas St E, Belleville, ON K8N 1E8, Canada</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Chef Basel Cuisine</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>(705) 748-2433</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2641 Television Rd, Peterborough, ON K9L 0E1, Canada</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Monday 3pm</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>(705) 748-2433</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2025-05-10</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Fresh Dreams</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>(705) 559-7731</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>373 Queen St, Peterborough, ON K9H 3J7, Canada</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no answer
+</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>(705) 559-7731</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2025-05-10</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Love You, Mean It - Bar &amp; Restaurant</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>(705) 742-6181</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>135 Hunter St W, Peterborough, ON K9H 2K7, Canada</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Copper Spoons</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>(705) 760-0541</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>540 Romaine St, Peterborough, ON K9J 2E2, Canada</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>THE RINK TAP AND GRILL</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>(705) 874-2935</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>597 Monaghan Rd, Peterborough, ON K9J 5J1, Canada</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Jack's Family Restaurant ~ Peterborough</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>(705) 740-9776</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>91 George St N, Peterborough, ON K9J 3G3, Canada</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Porch &amp; Pint Pub</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>(705) 750-0598</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>172 Lansdowne St E, Peterborough, ON K9J 7N9, Canada</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interested  
+Said will callback Wednesday
+Quote 500$ -------- callback Thursday
+</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>(705) 750-0598</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2025-05-12</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Erben</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>(705) 874-8379</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>379 George St N, Peterborough, ON K9H 3R2, Canada</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Turnbull Cafe</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>(705) 775-2233</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>170 Simcoe St, Peterborough, ON K9H 2H7, Canada</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seb call back
+</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>(705) 775-2233</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2025-05-12</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>The Speak Easy Cafe</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>(705) 749-9589</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>362 George St N, Peterborough, ON K9H 2H6, Canada</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Fifties Good Time Cafe</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>(705) 741-3812</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>590 Monaghan Rd, Peterborough, ON K9J 5H9, Canada</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>CC’s Café</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>(705) 775-7005</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>833 Chemong Rd, Peterborough, ON K9H 5Z5, Canada</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Cambodian Village Restaurant</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>called</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>(613) 536-0426</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>347 King St E, Kingston, ON K7L 3B5, Canada</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>call back june</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>(613) 536-0426</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2025-05-12</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Miss Bāo Restaurant + Cocktail Bar</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>(613) 545-0123</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>286 Princess St, Kingston, ON K7L 1B5, Canada</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Morrison's Restaurant</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>(613) 542-9483</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>318 King St E, Kingston, ON K7L 2Z3, Canada</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>(613) 542-9483</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Kingston Coffee House</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>(613) 531-7994</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>322 King St E, Kingston, ON K7L 3B4, Canada</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Chit Chat Café</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>(613) 777-8565</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>172 Ontario St, Kingston, ON K7L 2Y8, Canada</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Coffee Way Donuts</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>(613) 546-9106</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>472 Division St, Kingston, ON K7K 4B1, Canada</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Coffee Trends and Mile and a Quarter Ice Cream</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>called</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>(613) 634-7377</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>772 Blackburn Mews, Kingston, ON K7P 2N7, Canada</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Said no but i didnt persuade them</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>(613) 634-7377</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2025-05-12</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Philo and Kero Cafe</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>called</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>(613) 544-2297</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>791 Princess St Unit 104, Kingston, ON K7L 1E9, Canada</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Bad english have seb callback</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>(613) 544-2297</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2025-05-12</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>CommUnity Café</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>100 Days Rd, Kingston, ON K7M 6T5, Canada</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Delightfully Different Tea Room</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>(613) 766-5966</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>197 Wellington St, Kingston, ON K7K 2Y6, Canada</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>M &amp; J Cakes &amp; Cookies cafee</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>(647) 938-8654</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>252 Ontario St, Kingston, ON K7L 5P7, Canada</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Big Bites Kingston</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>(613) 766-0114</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>900 Montreal St, Kingston, ON K7K 3J9, Canada</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Hoagie House</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>(613) 542-5971</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>384 Division St, Kingston, ON K7K 4A5, Canada</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Seoul 2 Soul</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>(613) 507-6777</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>282 Princess St, Kingston, ON K7L 1B5, Canada</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Chez Lucien</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>(613) 241-3533</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>137 Murray St, Ottawa, ON K1N 5M7, Canada</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Call for owner around 10am</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2025-05-12</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>The Koven</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>called</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>(613) 422-5666</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>93 Murray St, Ottawa, ON K1N 5M6, Canada</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seb call and ask to send examples via email
+</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2025-05-12</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Ceasar Rosa's U-Rock Cafe</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>986 Wellington St. W, Ottawa, ON K1Y 2X8, Canada</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Le Moulin de Provence KD METCALFE &amp; QUEEN</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>callback</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>(613) 695-2253</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>30 Metcalfe St, Ottawa, ON K1P 5L4, Canada</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">callback before 2pm
+</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>2025-05-12</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Café des Tours</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>385 Sussex Dr, Ottawa, ON K1N 1J9, Canada</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Hugo Café</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>(613) 230-0084</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>399 Bank St, Ottawa, ON K2P 1Y3, Canada</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Café Qui Pense</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>204 Main St, Ottawa, ON K1S 0G4, Canada</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>DeliKat Café</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>(613) 235-7232</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>277 Sparks St., Ottawa, ON K1R 7X9, Canada</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Babylonia Cafe</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>(613) 728-1449</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>1319 Shillington Ave, Ottawa, ON K1Z 8A3, Canada</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Casa di Moni Café and Gelato</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>(613) 789-7172</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>51 York St, Ottawa, ON K1N 9B7, Canada</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Mellos Coffee Shop</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>(613) 224-6411</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>1516 Merivale Rd, Nepean, ON K2E 5P3, Canada</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Nepean</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Wilf &amp; Ada's (No reservations)</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>(613) 231-7959</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>510 Bank St, Ottawa, ON K2P 1C1, Canada</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Cozy's Express</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>(613) 746-2930</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>1572 Michael St, Ottawa, ON K1B 3T7, Canada</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Meadows Diner</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>(613) 567-5214</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>455 Preston St, Ottawa, ON K1S 3L2, Canada</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Bramasole Diner</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>tocall</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>(613) 234-0502</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>428 Bank St, Ottawa, ON K2P 1Y8, Canada</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>